<commit_message>
Initial VMware operations tool release
</commit_message>
<xml_diff>
--- a/templates/distributed_switch.xlsx
+++ b/templates/distributed_switch.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="分布式交换机" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="分布式端口组" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="批量数据" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="使用说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'批量数据'!$A$1:$D$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,16 +28,50 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="00EAF2FF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00EAF2FF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009FDBFF"/>
+    </font>
+    <font>
+      <color rgb="00B9C7DA"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0020324D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F1726"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0013233A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +79,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00304B6E"/>
+      </left>
+      <right style="thin">
+        <color rgb="00304B6E"/>
+      </right>
+      <top style="thin">
+        <color rgb="00304B6E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00304B6E"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,27 +482,45 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>VC</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>数据中心</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>分布式交换机名称</t>
-        </is>
-      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>交换机名称</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>上行链路数</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -445,32 +531,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>分布式交换机模板</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>使用提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>• 在第一张表中填写待创建的分布式交换机数据。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>• 必填列：VC、数据中心、交换机名称。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>• 上行链路数留空时，程序会按默认值执行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>字段列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>VC</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>分布式交换机名称</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>端口组名称</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>端口组VLAN</t>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>数据中心</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>交换机名称</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>上行链路数</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>